<commit_message>
Ontology.xlsx：Equal〜SubsetOf に builtInFunction の値を書く（plrDart 追記R604）
- G93:G99 の右に「| builtInFunction」と値（equal・greaterEqual・greaterThan・times・plus・divide・subsetOf。Dart の enum BuiltIn の要素名）
- CI の cto.pl を osspublish の MR !2（「| 属性」カラム）のコミットにする。マージされたら dev のコミットに戻す

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/ontology/Ontology.xlsx
+++ b/ontology/Ontology.xlsx
@@ -1473,7 +1473,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="14" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="141">
+  <cellXfs count="143">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
@@ -1896,6 +1896,12 @@
     </xf>
     <xf numFmtId="0" fontId="3" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="11" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf applyFill="1" numFmtId="0" fontId="6" fillId="11" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -3720,8 +3726,16 @@
           <t xml:space="preserve">Equal =</t>
         </is>
       </c>
-      <c r="H93" s="27"/>
-      <c r="I93" s="6"/>
+      <c r="H93" s="141" t="inlineStr">
+        <is>
+          <t xml:space="preserve">| builtInFunction</t>
+        </is>
+      </c>
+      <c r="I93" s="142" t="inlineStr">
+        <is>
+          <t xml:space="preserve">equal</t>
+        </is>
+      </c>
       <c r="J93" s="6"/>
     </row>
     <row r="94" spans="1:11" ht="34.799999999999997" customHeight="1">
@@ -3736,8 +3750,16 @@
           <t xml:space="preserve">GreaterEqual ≧</t>
         </is>
       </c>
-      <c r="H94" s="27"/>
-      <c r="I94" s="6"/>
+      <c r="H94" s="141" t="inlineStr">
+        <is>
+          <t xml:space="preserve">| builtInFunction</t>
+        </is>
+      </c>
+      <c r="I94" s="142" t="inlineStr">
+        <is>
+          <t xml:space="preserve">greaterEqual</t>
+        </is>
+      </c>
       <c r="J94" s="6"/>
     </row>
     <row r="95" spans="1:11" ht="34.799999999999997" customHeight="1">
@@ -3752,8 +3774,16 @@
           <t xml:space="preserve">GreaterThan &gt;</t>
         </is>
       </c>
-      <c r="H95" s="27"/>
-      <c r="I95" s="6"/>
+      <c r="H95" s="141" t="inlineStr">
+        <is>
+          <t xml:space="preserve">| builtInFunction</t>
+        </is>
+      </c>
+      <c r="I95" s="142" t="inlineStr">
+        <is>
+          <t xml:space="preserve">greaterThan</t>
+        </is>
+      </c>
       <c r="J95" s="6"/>
     </row>
     <row r="96" spans="1:11" ht="34.799999999999997" customHeight="1">
@@ -3768,8 +3798,16 @@
           <t xml:space="preserve">Times ×</t>
         </is>
       </c>
-      <c r="H96" s="27"/>
-      <c r="I96" s="6"/>
+      <c r="H96" s="141" t="inlineStr">
+        <is>
+          <t xml:space="preserve">| builtInFunction</t>
+        </is>
+      </c>
+      <c r="I96" s="142" t="inlineStr">
+        <is>
+          <t xml:space="preserve">times</t>
+        </is>
+      </c>
       <c r="J96" s="6"/>
     </row>
     <row r="97" spans="1:11" ht="34.799999999999997" customHeight="1">
@@ -3784,8 +3822,16 @@
           <t xml:space="preserve">Plus +</t>
         </is>
       </c>
-      <c r="H97" s="27"/>
-      <c r="I97" s="6"/>
+      <c r="H97" s="141" t="inlineStr">
+        <is>
+          <t xml:space="preserve">| builtInFunction</t>
+        </is>
+      </c>
+      <c r="I97" s="142" t="inlineStr">
+        <is>
+          <t xml:space="preserve">plus</t>
+        </is>
+      </c>
       <c r="J97" s="6"/>
     </row>
     <row r="98" spans="1:11" ht="34.799999999999997" customHeight="1">
@@ -3800,8 +3846,16 @@
           <t xml:space="preserve">Divide ÷</t>
         </is>
       </c>
-      <c r="H98" s="27"/>
-      <c r="I98" s="6"/>
+      <c r="H98" s="141" t="inlineStr">
+        <is>
+          <t xml:space="preserve">| builtInFunction</t>
+        </is>
+      </c>
+      <c r="I98" s="142" t="inlineStr">
+        <is>
+          <t xml:space="preserve">divide</t>
+        </is>
+      </c>
       <c r="J98" s="6"/>
     </row>
     <row r="99" spans="1:11" ht="34.799999999999997" customHeight="1">
@@ -3816,8 +3870,16 @@
           <t xml:space="preserve">SubsetOf ⊆</t>
         </is>
       </c>
-      <c r="H99" s="27"/>
-      <c r="I99" s="6"/>
+      <c r="H99" s="141" t="inlineStr">
+        <is>
+          <t xml:space="preserve">| builtInFunction</t>
+        </is>
+      </c>
+      <c r="I99" s="142" t="inlineStr">
+        <is>
+          <t xml:space="preserve">subsetOf</t>
+        </is>
+      </c>
       <c r="J99" s="6"/>
     </row>
     <row r="100" spans="1:11" ht="34.799999999999997" customHeight="1">

</xml_diff>